<commit_message>
feat(manager): enhance product variant excel import, order status filters, and manager product modal UI
</commit_message>
<xml_diff>
--- a/donhang_chieu_31_07/import_template.xlsx
+++ b/donhang_chieu_31_07/import_template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:M4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,33 +407,36 @@
         <v>Tên sản phẩm</v>
       </c>
       <c r="C1" t="str">
+        <v>Phân loại</v>
+      </c>
+      <c r="D1" t="str">
         <v>Danh mục</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Thương hiệu</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Đơn vị tính</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Giá nhập</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Giá bán</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Giá khuyến mãi</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Số lượng nhập</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>Loài mục tiêu</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Thông số kỹ thuật</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>Mô tả</v>
       </c>
     </row>
@@ -445,77 +448,124 @@
         <v>Luoc chai long tu dong cho thu cung</v>
       </c>
       <c r="C2" t="str">
+        <v>Size M</v>
+      </c>
+      <c r="D2" t="str">
         <v>GROOMING</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>FurCare</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>cái</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>60000</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>135000</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>109000</v>
       </c>
-      <c r="I2">
+      <c r="J2">
         <v>10</v>
       </c>
-      <c r="J2" t="str">
+      <c r="K2" t="str">
         <v>ALL</v>
       </c>
-      <c r="K2" t="str">
+      <c r="L2" t="str">
         <v>Màu sắc: Hồng, Kích thước: Trung bình, Chất liệu: Nhựa &amp; Thép</v>
       </c>
-      <c r="L2" t="str">
+      <c r="M2" t="str">
         <v>Lược chải lông tự động cho chó mèo.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v>128222</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Luoc chai long tu dong cho thu cung</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Size S</v>
+      </c>
+      <c r="D3" t="str">
+        <v>GROOMING</v>
+      </c>
+      <c r="E3" t="str">
+        <v>FurCare</v>
+      </c>
+      <c r="F3" t="str">
+        <v>cái</v>
+      </c>
+      <c r="G3">
+        <v>55000</v>
+      </c>
+      <c r="H3">
+        <v>120000</v>
+      </c>
+      <c r="I3">
+        <v>99000</v>
+      </c>
+      <c r="J3">
+        <v>15</v>
+      </c>
+      <c r="K3" t="str">
+        <v>ALL</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Màu sắc: Xanh, Kích thước: Nhỏ, Chất liệu: Nhựa &amp; Thép</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Lược chải lông tự động cho chó mèo.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
         <v>999999</v>
       </c>
-      <c r="B3" t="str">
+      <c r="B4" t="str">
         <v>Sản phẩm thử nghiệm mới Excel</v>
       </c>
-      <c r="C3" t="str">
+      <c r="C4" t="str">
+        <v>Hộp 500g</v>
+      </c>
+      <c r="D4" t="str">
         <v>ACCESSORY</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E4" t="str">
         <v>PetBrand</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F4" t="str">
         <v>cái</v>
       </c>
-      <c r="F3">
+      <c r="G4">
         <v>50000</v>
       </c>
-      <c r="G3">
+      <c r="H4">
         <v>100000</v>
       </c>
-      <c r="H3" t="str">
+      <c r="I4" t="str">
         <v/>
       </c>
-      <c r="I3">
+      <c r="J4">
         <v>20</v>
       </c>
-      <c r="J3" t="str">
+      <c r="K4" t="str">
         <v>CAT</v>
       </c>
-      <c r="K3" t="str">
+      <c r="L4" t="str">
         <v>Chất liệu: Cotton, Độ bền: Cao</v>
       </c>
-      <c r="L3" t="str">
+      <c r="M4" t="str">
         <v>Sản phẩm test tạo mới hoàn toàn từ file Excel.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>